<commit_message>
Add sensor statistics backfill functionality and update documentation
</commit_message>
<xml_diff>
--- a/db/init/data/db_init_data.xlsx
+++ b/db/init/data/db_init_data.xlsx
@@ -2,27 +2,27 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="R0ef3e4eba8f4401f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataSources" sheetId="2" r:id="R9f9e70a1b6aa4c52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UserTypes" sheetId="3" r:id="R7b27192156a54c0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductTypes" sheetId="4" r:id="R8e003c8b71d64f80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="5" r:id="R789fb37c8d5e4e74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MeasurementTypes" sheetId="6" r:id="R67ae668b3f924db0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SensorTypes" sheetId="7" r:id="R6bfc3cc9657b4665"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensors" sheetId="8" r:id="Rd227e1844c9b4965"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProcessConfigurations" sheetId="9" r:id="R291a78849fd548d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProcessSteps" sheetId="10" r:id="R3e25ea1678d14ea5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetProcessSteps" sheetId="11" r:id="R74d3e79694b745bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="12" r:id="Rf33491333d5f440a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FailureTypes" sheetId="13" r:id="R9024312df74645d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetFailureTypes" sheetId="14" r:id="R894e0ea01395479f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SensorFailureTypes" sheetId="15" r:id="R29ae7c2ca5b7497b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SensorStatistics" sheetId="16" r:id="R4e73b02a47894c30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="17" r:id="R34f8a067e7b841e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EtaBetas" sheetId="18" r:id="R200c0a07be664f9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gammas" sheetId="19" r:id="Ra3c92b410bf24ecc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetWorksheetLists" sheetId="20" r:id="Re30f805b294c40e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OperationsDoneLists" sheetId="21" r:id="R64879dbd88f1416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="R482fb45829de4ce3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataSources" sheetId="2" r:id="Rb4ed87190fb04faa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UserTypes" sheetId="3" r:id="R43d4df43e0844276"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductTypes" sheetId="4" r:id="Rc83434442e244475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="5" r:id="R5f022e0fe1114bc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MeasurementTypes" sheetId="6" r:id="Rbacc898a1aa34992"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SensorTypes" sheetId="7" r:id="R5e1e96f411f0437c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensors" sheetId="8" r:id="R6bfe5f8b511c4a90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProcessConfigurations" sheetId="9" r:id="R77c83382c02240f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProcessSteps" sheetId="10" r:id="R0bf704af0b574cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetProcessSteps" sheetId="11" r:id="R519da7b6d81c49aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="12" r:id="R54c595c8febd4b6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FailureTypes" sheetId="13" r:id="R22d59d7608a54b39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetFailureTypes" sheetId="14" r:id="R4c5c1604c1ad4ace"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SensorFailureTypes" sheetId="15" r:id="R1fdeef49b55843ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SensorStatistics" sheetId="16" r:id="R05e513fee2d04ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="17" r:id="R14a7ba8152544c4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EtaBetas" sheetId="18" r:id="R2b7c2dbb4d714d0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gammas" sheetId="19" r:id="R58c7bf371e5842f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetWorksheetLists" sheetId="20" r:id="R310eff81984348ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OperationsDoneLists" sheetId="21" r:id="Rb6e1fceb918d4f49"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -599,7 +599,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -609,6 +609,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -643,7 +648,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="41">
+  <x:cellXfs count="47">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="general"/>
@@ -770,6 +775,16 @@
     <x:xf numFmtId="204" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="204" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -881,7 +896,7 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="SensorStatisticsTable" displayName="SensorStatisticsTable" ref="A4:E10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="SensorStatisticsTable" displayName="SensorStatisticsTable" ref="A4:E7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="sensor_statistic_key"/>
     <x:tableColumn id="2" name="sensor_key"/>
@@ -1458,7 +1473,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa21dfc16721424a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ac9c710609f4c5d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1613,7 +1628,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R655a6fa0a58e48a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc60eada9227a4ee9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1768,7 +1783,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda5563890dca4bea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R493bd744d51d4d1b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1934,7 +1949,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc5c1b78b034941ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf31944879b524045"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2026,7 +2041,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R098f95274ae846fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31298f6a71ea459e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2167,7 +2182,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59abf497f6cf4043"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5acd09d49da14f9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2761,7 +2776,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f692e2a8995404f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7368b213861465f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2770,10 +2785,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="21" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="21" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -2783,128 +2798,98 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="33" t="str">
+      <x:c r="A4" s="46" t="str">
         <x:v>sensor_statistic_key</x:v>
       </x:c>
-      <x:c r="B4" s="33" t="str">
+      <x:c r="B4" s="46" t="str">
         <x:v>sensor_key</x:v>
       </x:c>
-      <x:c r="C4" s="33" t="str">
+      <x:c r="C4" s="46" t="str">
         <x:v>standard_deviation_value</x:v>
       </x:c>
-      <x:c r="D4" s="33" t="str">
+      <x:c r="D4" s="46" t="str">
         <x:v>average_value</x:v>
       </x:c>
-      <x:c r="E4" s="33" t="str">
+      <x:c r="E4" s="46" t="str">
         <x:v>learning_time</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="34" t="str">
+      <x:c r="A5" s="28" t="str">
         <x:v>sensor_stat_1</x:v>
       </x:c>
-      <x:c r="B5" s="34" t="str">
-        <x:v>tray_in_vqc</x:v>
-      </x:c>
-      <x:c r="C5" s="39" t="n">
-        <x:v>0.45</x:v>
-      </x:c>
-      <x:c r="D5" s="39" t="n">
-        <x:v>26.4</x:v>
-      </x:c>
-      <x:c r="E5" s="38" t="n">
-        <x:v>45992</x:v>
+      <x:c r="B5" s="28" t="str">
+        <x:v>tray_in_vqc</x:v>
+      </x:c>
+      <x:c r="C5" s="41" t="n">
+        <x:v>11.529079565464569</x:v>
+      </x:c>
+      <x:c r="D5" s="41" t="n">
+        <x:v>29.192629563265918</x:v>
+      </x:c>
+      <x:c r="E5" s="42" t="n">
+        <x:v>46033</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="34" t="str">
+      <x:c r="A6" s="28" t="str">
         <x:v>sensor_stat_2</x:v>
       </x:c>
-      <x:c r="B6" s="34" t="str">
-        <x:v>tray_out_vqc</x:v>
-      </x:c>
-      <x:c r="C6" s="39" t="n">
-        <x:v>1.1</x:v>
-      </x:c>
-      <x:c r="D6" s="39" t="n">
-        <x:v>104.5</x:v>
-      </x:c>
-      <x:c r="E6" s="38" t="n">
-        <x:v>45992</x:v>
+      <x:c r="B6" s="28" t="str">
+        <x:v>tray_out_vqc</x:v>
+      </x:c>
+      <x:c r="C6" s="41" t="n">
+        <x:v>5.866151139048425</x:v>
+      </x:c>
+      <x:c r="D6" s="41" t="n">
+        <x:v>109.8444798173757</x:v>
+      </x:c>
+      <x:c r="E6" s="42" t="n">
+        <x:v>46033</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="34" t="str">
+      <x:c r="A7" s="28" t="str">
         <x:v>sensor_stat_3</x:v>
       </x:c>
-      <x:c r="B7" s="34" t="str">
+      <x:c r="B7" s="28" t="str">
         <x:v>cylinder_status_vqc</x:v>
       </x:c>
-      <x:c r="C7" s="39" t="n">
-        <x:v>0.35</x:v>
-      </x:c>
-      <x:c r="D7" s="39" t="n">
-        <x:v>1.8</x:v>
-      </x:c>
-      <x:c r="E7" s="38" t="n">
-        <x:v>45992</x:v>
+      <x:c r="C7" s="41" t="n">
+        <x:v>2.8829210693675886</x:v>
+      </x:c>
+      <x:c r="D7" s="41" t="n">
+        <x:v>0.10196266102731127</x:v>
+      </x:c>
+      <x:c r="E7" s="42" t="n">
+        <x:v>46033</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="34" t="str">
-        <x:v>sensor_stat_4</x:v>
-      </x:c>
-      <x:c r="B8" s="34" t="str">
-        <x:v>tray_in_vqc</x:v>
-      </x:c>
-      <x:c r="C8" s="39" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="D8" s="39" t="n">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E8" s="38" t="n">
-        <x:v>46023</x:v>
-      </x:c>
+      <x:c r="A8"/>
+      <x:c r="B8"/>
+      <x:c r="C8"/>
+      <x:c r="D8"/>
+      <x:c r="E8"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="34" t="str">
-        <x:v>sensor_stat_5</x:v>
-      </x:c>
-      <x:c r="B9" s="34" t="str">
-        <x:v>tray_out_vqc</x:v>
-      </x:c>
-      <x:c r="C9" s="39" t="n">
-        <x:v>1.2</x:v>
-      </x:c>
-      <x:c r="D9" s="39" t="n">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="E9" s="38" t="n">
-        <x:v>46023</x:v>
-      </x:c>
+      <x:c r="A9"/>
+      <x:c r="B9"/>
+      <x:c r="C9"/>
+      <x:c r="D9"/>
+      <x:c r="E9"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="34" t="str">
-        <x:v>sensor_stat_6</x:v>
-      </x:c>
-      <x:c r="B10" s="34" t="str">
-        <x:v>cylinder_status_vqc</x:v>
-      </x:c>
-      <x:c r="C10" s="39" t="n">
-        <x:v>0.3</x:v>
-      </x:c>
-      <x:c r="D10" s="39" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="E10" s="38" t="n">
-        <x:v>46023</x:v>
-      </x:c>
+      <x:c r="A10"/>
+      <x:c r="B10"/>
+      <x:c r="C10"/>
+      <x:c r="D10"/>
+      <x:c r="E10"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a421b4abc1748a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d58d079bec14556"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -51905,7 +51890,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8023d149e9b447b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R731a5f43bcc74464"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -52014,7 +51999,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R165e6a0ec9e24009"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcd31f1998de44ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -52922,7 +52907,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7120c790d51f44c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R442b0288a3c64f30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -52988,7 +52973,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd98ceaf059d4df5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88298fb7a5b24f76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53189,7 +53174,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1735e23611bb4390"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18b21a9c2ab24248"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53604,7 +53589,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9e1949612264f11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68346f0f2bc74451"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53690,7 +53675,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9cd37de3f39483d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7523e6f988904a62"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53779,7 +53764,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ba1db084ad5464c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0c510b057514557"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53901,7 +53886,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3bdb8725b04739"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R700a9d3701954b39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54025,7 +54010,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red272f975a5d4467"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad61af5a0b0c4cb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54181,7 +54166,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cd8779eb4394100"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd61d4cd5d1d74a63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54635,7 +54620,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd32de329421c4c00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R192ea96fd41b4711"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54707,7 +54692,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R123bd97a9d3d4500"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf438a4aaafab4af3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor prediction parameter initialization and update database schema constraints
</commit_message>
<xml_diff>
--- a/db/init/data/db_init_data.xlsx
+++ b/db/init/data/db_init_data.xlsx
@@ -2,27 +2,27 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="Rf3b1ac2db5bd422b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataSources" sheetId="2" r:id="Redc02cc9964c447f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UserTypes" sheetId="3" r:id="Rc6762db6bcf748eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductTypes" sheetId="4" r:id="R663a36f4fba14a8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="5" r:id="R8c10932bfba8435c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MeasurementTypes" sheetId="6" r:id="Rd645ef9d1e164e89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SensorTypes" sheetId="7" r:id="Rfdcb3886124842ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensors" sheetId="8" r:id="R4e96f52cbd8143b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProcessConfigurations" sheetId="9" r:id="R630929e9fa594777"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProcessSteps" sheetId="10" r:id="R10b912e61756471f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetProcessSteps" sheetId="11" r:id="R1ca6cc0dbb004035"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="12" r:id="Rec0f4356c4db479c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FailureTypes" sheetId="13" r:id="Rf7e7192dbad8442a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetFailureTypes" sheetId="14" r:id="Rdc4df7808f734ce5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SensorFailureTypes" sheetId="15" r:id="Rb622adab754342a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SensorStatistics" sheetId="16" r:id="R96cec2f42ce44d52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="17" r:id="R5630d9e8353448d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EtaBetas" sheetId="18" r:id="Rfd50da0157f64239"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gammas" sheetId="19" r:id="Ree788c607bc14182"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetWorksheetLists" sheetId="20" r:id="Rd3977d81fa784ef6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OperationsDoneLists" sheetId="21" r:id="R69f26827900a4b28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="Rf157187309dc43a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataSources" sheetId="2" r:id="Rf5692f60d6ac4cbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UserTypes" sheetId="3" r:id="Ra7864075f7da4eec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProductTypes" sheetId="4" r:id="Ra84dc3076d374f43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="5" r:id="R12c606381a7044cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MeasurementTypes" sheetId="6" r:id="Red218458e15a4a65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SensorTypes" sheetId="7" r:id="R890b02d833474bd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensors" sheetId="8" r:id="R77eb355340954525"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProcessConfigurations" sheetId="9" r:id="R88d11315c0784f22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ProcessSteps" sheetId="10" r:id="R49197d5bee774a04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetProcessSteps" sheetId="11" r:id="Rff4601b8d505430f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Routing" sheetId="12" r:id="R8c7df934df5e489b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FailureTypes" sheetId="13" r:id="R0ed26f981a4c4b6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetFailureTypes" sheetId="14" r:id="R71e9365702224180"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SensorFailureTypes" sheetId="15" r:id="R59a326ebadac4fb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SensorStatistics" sheetId="16" r:id="R31fb48ca8bbf430f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="17" r:id="R6d6836520a1c4797"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EtaBetas" sheetId="18" r:id="R854d5264e22d40e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gammas" sheetId="19" r:id="R314922f5f5cb4473"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssetWorksheetLists" sheetId="20" r:id="R49e2e67b6aba4892"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OperationsDoneLists" sheetId="21" r:id="Rf03aa0dbdabb4e66"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -58,9 +58,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">External IDs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">cmms_asset_id, dc_asset_id and metric_function_id are prepared for future mappings and may remain blank for now.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Processing time</x:t>
@@ -648,7 +645,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="general"/>
@@ -784,6 +781,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1390,12 +1393,12 @@
       <x:c r="E8" s="1"/>
       <x:c r="F8" s="1"/>
     </x:row>
-    <x:row r="9" ht="18.75" customHeight="1">
-      <x:c r="A9" s="3" t="s">
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="47" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B9" s="25" t="s">
-        <x:v>10</x:v>
+      <x:c r="B9" s="47" t="str">
+        <x:v>cmms_asset_id and dc_asset_id connect the internal asset to CMMS and Data Collector identifiers. metric_function_id identifies the Data Collector metric. Blank seed values do not erase existing runtime mappings.</x:v>
       </x:c>
       <x:c r="C9" s="1"/>
       <x:c r="D9" s="1"/>
@@ -1404,10 +1407,10 @@
     </x:row>
     <x:row r="10" ht="18.75" customHeight="1">
       <x:c r="A10" s="3" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B10" s="25" t="s">
         <x:v>11</x:v>
-      </x:c>
-      <x:c r="B10" s="25" t="s">
-        <x:v>12</x:v>
       </x:c>
       <x:c r="C10" s="1"/>
       <x:c r="D10" s="1"/>
@@ -1416,10 +1419,10 @@
     </x:row>
     <x:row r="11" ht="18.75" customHeight="1">
       <x:c r="A11" s="3" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B11" s="25" t="s">
         <x:v>13</x:v>
-      </x:c>
-      <x:c r="B11" s="25" t="s">
-        <x:v>14</x:v>
       </x:c>
       <x:c r="C11" s="1"/>
       <x:c r="D11" s="1"/>
@@ -1428,22 +1431,22 @@
     </x:row>
     <x:row r="12" ht="18.75" customHeight="1">
       <x:c r="A12" s="3" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B12" s="25" t="s">
         <x:v>15</x:v>
-      </x:c>
-      <x:c r="B12" s="25" t="s">
-        <x:v>16</x:v>
       </x:c>
       <x:c r="C12" s="1"/>
       <x:c r="D12" s="1"/>
       <x:c r="E12" s="1"/>
       <x:c r="F12" s="1"/>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
+    <x:row r="13" ht="40" customHeight="1">
+      <x:c r="A13" s="48" t="str">
         <x:v>Prediction inputs</x:v>
       </x:c>
-      <x:c r="B13" t="str">
-        <x:v>Prediction-module input data is stored on the FailureTypes through OperationsDoneLists sheets.</x:v>
+      <x:c r="B13" s="48" t="str">
+        <x:v>Static sensor and maintenance inputs remain in the workbook. Failure types, asset/sensor failure relations and their cold-start parameters are created at runtime from CMMS data.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1454,12 +1457,12 @@
         <x:v>Attached asset IDs 1/2 map to visual_qc/preparation; sensor IDs 1/2/3 map to tray_in_vqc/tray_out_vqc/cylinder_status_vqc.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
+    <x:row r="15" ht="46" customHeight="1">
+      <x:c r="A15" s="48" t="str">
         <x:v>Initial parameters</x:v>
       </x:c>
-      <x:c r="B15" t="str">
-        <x:v>Eta/Beta and Gamma rows contain dummy initial values. The prediction module may update or append learned values while running.</x:v>
+      <x:c r="B15" s="48" t="str">
+        <x:v>Failure types and their asset/sensor relations are created from CMMS data at runtime. Eta/Beta and Gamma cold-start defaults are inserted only when a new relation has no parameter history; later values belong to the prediction module.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1473,7 +1476,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refb59c1d60754eb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7c263bf24344d36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1494,7 +1497,7 @@
     </x:row>
     <x:row r="2" ht="18.75" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="7"/>
@@ -1506,21 +1509,21 @@
     </x:row>
     <x:row r="4" ht="26.100000381469727" customHeight="1">
       <x:c r="A4" s="3" t="s">
+        <x:v>151</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
         <x:v>152</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="s">
+      <x:c r="C4" s="7" t="s">
         <x:v>153</x:v>
-      </x:c>
-      <x:c r="C4" s="7" t="s">
-        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="18.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
         <x:v>155</x:v>
-      </x:c>
-      <x:c r="B5" s="3" t="s">
-        <x:v>156</x:v>
       </x:c>
       <x:c r="C5" s="9">
         <x:v>0</x:v>
@@ -1528,10 +1531,10 @@
     </x:row>
     <x:row r="6" ht="18.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
+        <x:v>156</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="s">
         <x:v>157</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="s">
-        <x:v>158</x:v>
       </x:c>
       <x:c r="C6" s="9">
         <x:v>60</x:v>
@@ -1539,10 +1542,10 @@
     </x:row>
     <x:row r="7" ht="18.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="s">
         <x:v>159</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="s">
-        <x:v>160</x:v>
       </x:c>
       <x:c r="C7" s="9">
         <x:v>5</x:v>
@@ -1550,10 +1553,10 @@
     </x:row>
     <x:row r="8" ht="18.75" customHeight="1">
       <x:c r="A8" s="3" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="s">
         <x:v>161</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="s">
-        <x:v>162</x:v>
       </x:c>
       <x:c r="C8" s="9">
         <x:v>30</x:v>
@@ -1561,10 +1564,10 @@
     </x:row>
     <x:row r="9" ht="18.75" customHeight="1">
       <x:c r="A9" s="3" t="s">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="s">
         <x:v>163</x:v>
-      </x:c>
-      <x:c r="B9" s="3" t="s">
-        <x:v>164</x:v>
       </x:c>
       <x:c r="C9" s="9">
         <x:v>50</x:v>
@@ -1572,10 +1575,10 @@
     </x:row>
     <x:row r="10" ht="18.75" customHeight="1">
       <x:c r="A10" s="3" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
-        <x:v>162</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="C10" s="9">
         <x:v>20</x:v>
@@ -1583,10 +1586,10 @@
     </x:row>
     <x:row r="11" ht="18.75" customHeight="1">
       <x:c r="A11" s="3" t="s">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="s">
         <x:v>166</x:v>
-      </x:c>
-      <x:c r="B11" s="3" t="s">
-        <x:v>167</x:v>
       </x:c>
       <x:c r="C11" s="9">
         <x:v>44</x:v>
@@ -1594,10 +1597,10 @@
     </x:row>
     <x:row r="12" ht="18.75" customHeight="1">
       <x:c r="A12" s="3" t="s">
-        <x:v>168</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
-        <x:v>162</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="C12" s="9">
         <x:v>20</x:v>
@@ -1605,10 +1608,10 @@
     </x:row>
     <x:row r="13" ht="18.75" customHeight="1">
       <x:c r="A13" s="3" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="B13" s="3" t="s">
         <x:v>169</x:v>
-      </x:c>
-      <x:c r="B13" s="3" t="s">
-        <x:v>170</x:v>
       </x:c>
       <x:c r="C13" s="9">
         <x:v>30</x:v>
@@ -1616,10 +1619,10 @@
     </x:row>
     <x:row r="14" ht="18.75" customHeight="1">
       <x:c r="A14" s="3" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="s">
         <x:v>171</x:v>
-      </x:c>
-      <x:c r="B14" s="3" t="s">
-        <x:v>172</x:v>
       </x:c>
       <x:c r="C14" s="9">
         <x:v>5</x:v>
@@ -1628,7 +1631,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc452495387e8423e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a051a3618964bb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1649,7 +1652,7 @@
     </x:row>
     <x:row r="2" ht="18.75" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>173</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -1661,129 +1664,129 @@
     </x:row>
     <x:row r="4" ht="26.100000381469727" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>144</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="18.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>155</x:v>
+        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="18.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="18.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>159</x:v>
+        <x:v>158</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="18.75" customHeight="1">
       <x:c r="A8" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>161</x:v>
+        <x:v>160</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="18.75" customHeight="1">
       <x:c r="A9" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>163</x:v>
+        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="18.75" customHeight="1">
       <x:c r="A10" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C10" s="3" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="18.75" customHeight="1">
       <x:c r="A11" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>166</x:v>
+        <x:v>165</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="18.75" customHeight="1">
       <x:c r="A12" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>168</x:v>
+        <x:v>167</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="18.75" customHeight="1">
       <x:c r="A13" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="18.75" customHeight="1">
       <x:c r="A14" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
-        <x:v>69</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>171</x:v>
+        <x:v>170</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64071f881e264654"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67fa90c5ca764d39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1804,7 +1807,7 @@
     </x:row>
     <x:row r="2" ht="18.75" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>174</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -1816,112 +1819,112 @@
     </x:row>
     <x:row r="4" ht="26.100000381469727" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>144</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>175</x:v>
+        <x:v>174</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="18.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>155</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="18.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>159</x:v>
+        <x:v>158</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="18.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
-        <x:v>159</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>161</x:v>
+        <x:v>160</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="18.75" customHeight="1">
       <x:c r="A8" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
-        <x:v>161</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>163</x:v>
+        <x:v>162</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="18.75" customHeight="1">
       <x:c r="A9" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
-        <x:v>163</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="18.75" customHeight="1">
       <x:c r="A10" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="s">
         <x:v>165</x:v>
-      </x:c>
-      <x:c r="C10" s="3" t="s">
-        <x:v>166</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="18.75" customHeight="1">
       <x:c r="A11" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
-        <x:v>166</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>168</x:v>
+        <x:v>167</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="18.75" customHeight="1">
       <x:c r="A12" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
+        <x:v>167</x:v>
+      </x:c>
+      <x:c r="C12" s="3" t="s">
         <x:v>168</x:v>
-      </x:c>
-      <x:c r="C12" s="3" t="s">
-        <x:v>169</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="18.75" customHeight="1">
       <x:c r="A13" s="3" t="s">
-        <x:v>149</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
-        <x:v>169</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>171</x:v>
+        <x:v>170</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1949,7 +1952,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec23b67637574245"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30bfcc5e6baf434f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1988,60 +1991,30 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
-      <x:c r="B5" s="34" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C5" s="34" t="str">
-        <x:v>Failure type 1</x:v>
-      </x:c>
-      <x:c r="D5" s="35" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E5" s="34" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="A5" s="34"/>
+      <x:c r="B5" s="34"/>
+      <x:c r="C5" s="34"/>
+      <x:c r="D5" s="34"/>
+      <x:c r="E5" s="34"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
-      <x:c r="B6" s="34" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C6" s="34" t="str">
-        <x:v>Failure type 2</x:v>
-      </x:c>
-      <x:c r="D6" s="35" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E6" s="34" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="A6" s="34"/>
+      <x:c r="B6" s="34"/>
+      <x:c r="C6" s="34"/>
+      <x:c r="D6" s="34"/>
+      <x:c r="E6" s="34"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
-      <x:c r="B7" s="34" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C7" s="34" t="str">
-        <x:v>Failure type 3</x:v>
-      </x:c>
-      <x:c r="D7" s="35" t="b">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E7" s="34" t="n">
-        <x:v>3</x:v>
-      </x:c>
+      <x:c r="A7" s="34"/>
+      <x:c r="B7" s="34"/>
+      <x:c r="C7" s="34"/>
+      <x:c r="D7" s="34"/>
+      <x:c r="E7" s="34"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cade5085a944286"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09601103f7484041"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2088,101 +2061,45 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="34" t="str">
-        <x:v>asset_failure_type_1</x:v>
-      </x:c>
-      <x:c r="B5" s="34" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C5" s="34" t="str">
-        <x:v>visual_qc</x:v>
-      </x:c>
-      <x:c r="D5" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
-      <x:c r="E5" s="36" t="n">
-        <x:v>0.1</x:v>
-      </x:c>
-      <x:c r="F5" s="37" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G5" s="34" t="n">
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="A5" s="34"/>
+      <x:c r="B5" s="34"/>
+      <x:c r="C5" s="34"/>
+      <x:c r="D5" s="34"/>
+      <x:c r="E5" s="36"/>
+      <x:c r="F5" s="37"/>
+      <x:c r="G5" s="34"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="34" t="str">
-        <x:v>asset_failure_type_2</x:v>
-      </x:c>
-      <x:c r="B6" s="34" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C6" s="34" t="str">
-        <x:v>visual_qc</x:v>
-      </x:c>
-      <x:c r="D6" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
-      <x:c r="E6" s="36" t="n">
-        <x:v>0.07</x:v>
-      </x:c>
-      <x:c r="F6" s="37" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G6" s="34" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="A6" s="34"/>
+      <x:c r="B6" s="34"/>
+      <x:c r="C6" s="34"/>
+      <x:c r="D6" s="34"/>
+      <x:c r="E6" s="36"/>
+      <x:c r="F6" s="37"/>
+      <x:c r="G6" s="34"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="34" t="str">
-        <x:v>asset_failure_type_3</x:v>
-      </x:c>
-      <x:c r="B7" s="34" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C7" s="34" t="str">
-        <x:v>preparation</x:v>
-      </x:c>
-      <x:c r="D7" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
-      <x:c r="E7" s="36" t="n">
-        <x:v>0.2</x:v>
-      </x:c>
-      <x:c r="F7" s="37" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G7" s="34" t="n">
-        <x:v>3</x:v>
-      </x:c>
+      <x:c r="A7" s="34"/>
+      <x:c r="B7" s="34"/>
+      <x:c r="C7" s="34"/>
+      <x:c r="D7" s="34"/>
+      <x:c r="E7" s="36"/>
+      <x:c r="F7" s="37"/>
+      <x:c r="G7" s="34"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="34" t="str">
-        <x:v>asset_failure_type_4</x:v>
-      </x:c>
-      <x:c r="B8" s="34" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C8" s="34" t="str">
-        <x:v>preparation</x:v>
-      </x:c>
-      <x:c r="D8" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
-      <x:c r="E8" s="36" t="n">
-        <x:v>0.05</x:v>
-      </x:c>
-      <x:c r="F8" s="37" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G8" s="34" t="n">
-        <x:v>4</x:v>
-      </x:c>
+      <x:c r="A8" s="34"/>
+      <x:c r="B8" s="34"/>
+      <x:c r="C8" s="34"/>
+      <x:c r="D8" s="34"/>
+      <x:c r="E8" s="36"/>
+      <x:c r="F8" s="37"/>
+      <x:c r="G8" s="34"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R428afc65e2c94186"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R309ba099698f40b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2213,570 +2130,264 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="34" t="str">
-        <x:v>tray_in_vqc__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B5" s="34" t="str">
-        <x:v>tray_in_vqc</x:v>
-      </x:c>
-      <x:c r="C5" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A5" s="34"/>
+      <x:c r="B5" s="34"/>
+      <x:c r="C5" s="34"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="34" t="str">
-        <x:v>tray_in_vqc__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B6" s="34" t="str">
-        <x:v>tray_in_vqc</x:v>
-      </x:c>
-      <x:c r="C6" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A6" s="34"/>
+      <x:c r="B6" s="34"/>
+      <x:c r="C6" s="34"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="34" t="str">
-        <x:v>tray_in_vqc__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B7" s="34" t="str">
-        <x:v>tray_in_vqc</x:v>
-      </x:c>
-      <x:c r="C7" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A7" s="34"/>
+      <x:c r="B7" s="34"/>
+      <x:c r="C7" s="34"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="34" t="str">
-        <x:v>tray_out_vqc__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B8" s="34" t="str">
-        <x:v>tray_out_vqc</x:v>
-      </x:c>
-      <x:c r="C8" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A8" s="34"/>
+      <x:c r="B8" s="34"/>
+      <x:c r="C8" s="34"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="34" t="str">
-        <x:v>tray_out_vqc__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B9" s="34" t="str">
-        <x:v>tray_out_vqc</x:v>
-      </x:c>
-      <x:c r="C9" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A9" s="34"/>
+      <x:c r="B9" s="34"/>
+      <x:c r="C9" s="34"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="34" t="str">
-        <x:v>tray_out_vqc__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B10" s="34" t="str">
-        <x:v>tray_out_vqc</x:v>
-      </x:c>
-      <x:c r="C10" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A10" s="34"/>
+      <x:c r="B10" s="34"/>
+      <x:c r="C10" s="34"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="34" t="str">
-        <x:v>cylinder_status_vqc__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B11" s="34" t="str">
-        <x:v>cylinder_status_vqc</x:v>
-      </x:c>
-      <x:c r="C11" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A11" s="34"/>
+      <x:c r="B11" s="34"/>
+      <x:c r="C11" s="34"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="34" t="str">
-        <x:v>cylinder_status_vqc__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B12" s="34" t="str">
-        <x:v>cylinder_status_vqc</x:v>
-      </x:c>
-      <x:c r="C12" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A12" s="34"/>
+      <x:c r="B12" s="34"/>
+      <x:c r="C12" s="34"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="34" t="str">
-        <x:v>cylinder_status_vqc__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B13" s="34" t="str">
-        <x:v>cylinder_status_vqc</x:v>
-      </x:c>
-      <x:c r="C13" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A13" s="34"/>
+      <x:c r="B13" s="34"/>
+      <x:c r="C13" s="34"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="34" t="str">
-        <x:v>tray_in_prep__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B14" s="34" t="str">
-        <x:v>tray_in_prep</x:v>
-      </x:c>
-      <x:c r="C14" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A14" s="34"/>
+      <x:c r="B14" s="34"/>
+      <x:c r="C14" s="34"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="34" t="str">
-        <x:v>tray_in_prep__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B15" s="34" t="str">
-        <x:v>tray_in_prep</x:v>
-      </x:c>
-      <x:c r="C15" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A15" s="34"/>
+      <x:c r="B15" s="34"/>
+      <x:c r="C15" s="34"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="34" t="str">
-        <x:v>tray_in_prep__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B16" s="34" t="str">
-        <x:v>tray_in_prep</x:v>
-      </x:c>
-      <x:c r="C16" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A16" s="34"/>
+      <x:c r="B16" s="34"/>
+      <x:c r="C16" s="34"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="34" t="str">
-        <x:v>tray_out_prep__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B17" s="34" t="str">
-        <x:v>tray_out_prep</x:v>
-      </x:c>
-      <x:c r="C17" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A17" s="34"/>
+      <x:c r="B17" s="34"/>
+      <x:c r="C17" s="34"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="34" t="str">
-        <x:v>tray_out_prep__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B18" s="34" t="str">
-        <x:v>tray_out_prep</x:v>
-      </x:c>
-      <x:c r="C18" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A18" s="34"/>
+      <x:c r="B18" s="34"/>
+      <x:c r="C18" s="34"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="34" t="str">
-        <x:v>tray_out_prep__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B19" s="34" t="str">
-        <x:v>tray_out_prep</x:v>
-      </x:c>
-      <x:c r="C19" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A19" s="34"/>
+      <x:c r="B19" s="34"/>
+      <x:c r="C19" s="34"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="34" t="str">
-        <x:v>cylinder_status_prep__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B20" s="34" t="str">
-        <x:v>cylinder_status_prep</x:v>
-      </x:c>
-      <x:c r="C20" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A20" s="34"/>
+      <x:c r="B20" s="34"/>
+      <x:c r="C20" s="34"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="34" t="str">
-        <x:v>cylinder_status_prep__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B21" s="34" t="str">
-        <x:v>cylinder_status_prep</x:v>
-      </x:c>
-      <x:c r="C21" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A21" s="34"/>
+      <x:c r="B21" s="34"/>
+      <x:c r="C21" s="34"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="34" t="str">
-        <x:v>cylinder_status_prep__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B22" s="34" t="str">
-        <x:v>cylinder_status_prep</x:v>
-      </x:c>
-      <x:c r="C22" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A22" s="34"/>
+      <x:c r="B22" s="34"/>
+      <x:c r="C22" s="34"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="34" t="str">
-        <x:v>tray_in_asb1__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B23" s="34" t="str">
-        <x:v>tray_in_asb1</x:v>
-      </x:c>
-      <x:c r="C23" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A23" s="34"/>
+      <x:c r="B23" s="34"/>
+      <x:c r="C23" s="34"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="34" t="str">
-        <x:v>tray_in_asb1__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B24" s="34" t="str">
-        <x:v>tray_in_asb1</x:v>
-      </x:c>
-      <x:c r="C24" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A24" s="34"/>
+      <x:c r="B24" s="34"/>
+      <x:c r="C24" s="34"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="34" t="str">
-        <x:v>tray_in_asb1__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B25" s="34" t="str">
-        <x:v>tray_in_asb1</x:v>
-      </x:c>
-      <x:c r="C25" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A25" s="34"/>
+      <x:c r="B25" s="34"/>
+      <x:c r="C25" s="34"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="34" t="str">
-        <x:v>tray_out_asb1__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B26" s="34" t="str">
-        <x:v>tray_out_asb1</x:v>
-      </x:c>
-      <x:c r="C26" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A26" s="34"/>
+      <x:c r="B26" s="34"/>
+      <x:c r="C26" s="34"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="34" t="str">
-        <x:v>tray_out_asb1__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B27" s="34" t="str">
-        <x:v>tray_out_asb1</x:v>
-      </x:c>
-      <x:c r="C27" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A27" s="34"/>
+      <x:c r="B27" s="34"/>
+      <x:c r="C27" s="34"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="34" t="str">
-        <x:v>tray_out_asb1__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B28" s="34" t="str">
-        <x:v>tray_out_asb1</x:v>
-      </x:c>
-      <x:c r="C28" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A28" s="34"/>
+      <x:c r="B28" s="34"/>
+      <x:c r="C28" s="34"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="34" t="str">
-        <x:v>cylinder_status_asb1__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B29" s="34" t="str">
-        <x:v>cylinder_status_asb1</x:v>
-      </x:c>
-      <x:c r="C29" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A29" s="34"/>
+      <x:c r="B29" s="34"/>
+      <x:c r="C29" s="34"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="34" t="str">
-        <x:v>cylinder_status_asb1__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B30" s="34" t="str">
-        <x:v>cylinder_status_asb1</x:v>
-      </x:c>
-      <x:c r="C30" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A30" s="34"/>
+      <x:c r="B30" s="34"/>
+      <x:c r="C30" s="34"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="34" t="str">
-        <x:v>cylinder_status_asb1__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B31" s="34" t="str">
-        <x:v>cylinder_status_asb1</x:v>
-      </x:c>
-      <x:c r="C31" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A31" s="34"/>
+      <x:c r="B31" s="34"/>
+      <x:c r="C31" s="34"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="34" t="str">
-        <x:v>tray_in_asb2__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B32" s="34" t="str">
-        <x:v>tray_in_asb2</x:v>
-      </x:c>
-      <x:c r="C32" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A32" s="34"/>
+      <x:c r="B32" s="34"/>
+      <x:c r="C32" s="34"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="34" t="str">
-        <x:v>tray_in_asb2__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B33" s="34" t="str">
-        <x:v>tray_in_asb2</x:v>
-      </x:c>
-      <x:c r="C33" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A33" s="34"/>
+      <x:c r="B33" s="34"/>
+      <x:c r="C33" s="34"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="34" t="str">
-        <x:v>tray_in_asb2__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B34" s="34" t="str">
-        <x:v>tray_in_asb2</x:v>
-      </x:c>
-      <x:c r="C34" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A34" s="34"/>
+      <x:c r="B34" s="34"/>
+      <x:c r="C34" s="34"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="34" t="str">
-        <x:v>tray_out_asb2__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B35" s="34" t="str">
-        <x:v>tray_out_asb2</x:v>
-      </x:c>
-      <x:c r="C35" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A35" s="34"/>
+      <x:c r="B35" s="34"/>
+      <x:c r="C35" s="34"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="34" t="str">
-        <x:v>tray_out_asb2__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B36" s="34" t="str">
-        <x:v>tray_out_asb2</x:v>
-      </x:c>
-      <x:c r="C36" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A36" s="34"/>
+      <x:c r="B36" s="34"/>
+      <x:c r="C36" s="34"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="34" t="str">
-        <x:v>tray_out_asb2__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B37" s="34" t="str">
-        <x:v>tray_out_asb2</x:v>
-      </x:c>
-      <x:c r="C37" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A37" s="34"/>
+      <x:c r="B37" s="34"/>
+      <x:c r="C37" s="34"/>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="34" t="str">
-        <x:v>cylinder_status_asb2__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B38" s="34" t="str">
-        <x:v>cylinder_status_asb2</x:v>
-      </x:c>
-      <x:c r="C38" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A38" s="34"/>
+      <x:c r="B38" s="34"/>
+      <x:c r="C38" s="34"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="34" t="str">
-        <x:v>cylinder_status_asb2__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B39" s="34" t="str">
-        <x:v>cylinder_status_asb2</x:v>
-      </x:c>
-      <x:c r="C39" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A39" s="34"/>
+      <x:c r="B39" s="34"/>
+      <x:c r="C39" s="34"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="34" t="str">
-        <x:v>cylinder_status_asb2__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B40" s="34" t="str">
-        <x:v>cylinder_status_asb2</x:v>
-      </x:c>
-      <x:c r="C40" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A40" s="34"/>
+      <x:c r="B40" s="34"/>
+      <x:c r="C40" s="34"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="34" t="str">
-        <x:v>global_temp__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B41" s="34" t="str">
-        <x:v>global_temp</x:v>
-      </x:c>
-      <x:c r="C41" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A41" s="34"/>
+      <x:c r="B41" s="34"/>
+      <x:c r="C41" s="34"/>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="34" t="str">
-        <x:v>global_temp__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B42" s="34" t="str">
-        <x:v>global_temp</x:v>
-      </x:c>
-      <x:c r="C42" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A42" s="34"/>
+      <x:c r="B42" s="34"/>
+      <x:c r="C42" s="34"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="34" t="str">
-        <x:v>global_temp__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B43" s="34" t="str">
-        <x:v>global_temp</x:v>
-      </x:c>
-      <x:c r="C43" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A43" s="34"/>
+      <x:c r="B43" s="34"/>
+      <x:c r="C43" s="34"/>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="34" t="str">
-        <x:v>global_hum__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B44" s="34" t="str">
-        <x:v>global_hum</x:v>
-      </x:c>
-      <x:c r="C44" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A44" s="34"/>
+      <x:c r="B44" s="34"/>
+      <x:c r="C44" s="34"/>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="34" t="str">
-        <x:v>global_hum__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B45" s="34" t="str">
-        <x:v>global_hum</x:v>
-      </x:c>
-      <x:c r="C45" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A45" s="34"/>
+      <x:c r="B45" s="34"/>
+      <x:c r="C45" s="34"/>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="34" t="str">
-        <x:v>global_hum__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B46" s="34" t="str">
-        <x:v>global_hum</x:v>
-      </x:c>
-      <x:c r="C46" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A46" s="34"/>
+      <x:c r="B46" s="34"/>
+      <x:c r="C46" s="34"/>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="34" t="str">
-        <x:v>protec_acceleration_x__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B47" s="34" t="str">
-        <x:v>protec_acceleration_x</x:v>
-      </x:c>
-      <x:c r="C47" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A47" s="34"/>
+      <x:c r="B47" s="34"/>
+      <x:c r="C47" s="34"/>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="34" t="str">
-        <x:v>protec_acceleration_x__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B48" s="34" t="str">
-        <x:v>protec_acceleration_x</x:v>
-      </x:c>
-      <x:c r="C48" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A48" s="34"/>
+      <x:c r="B48" s="34"/>
+      <x:c r="C48" s="34"/>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="34" t="str">
-        <x:v>protec_acceleration_x__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B49" s="34" t="str">
-        <x:v>protec_acceleration_x</x:v>
-      </x:c>
-      <x:c r="C49" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A49" s="34"/>
+      <x:c r="B49" s="34"/>
+      <x:c r="C49" s="34"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="34" t="str">
-        <x:v>protec_acceleration_y__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B50" s="34" t="str">
-        <x:v>protec_acceleration_y</x:v>
-      </x:c>
-      <x:c r="C50" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A50" s="34"/>
+      <x:c r="B50" s="34"/>
+      <x:c r="C50" s="34"/>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="34" t="str">
-        <x:v>protec_acceleration_y__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B51" s="34" t="str">
-        <x:v>protec_acceleration_y</x:v>
-      </x:c>
-      <x:c r="C51" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A51" s="34"/>
+      <x:c r="B51" s="34"/>
+      <x:c r="C51" s="34"/>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="34" t="str">
-        <x:v>protec_acceleration_y__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B52" s="34" t="str">
-        <x:v>protec_acceleration_y</x:v>
-      </x:c>
-      <x:c r="C52" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A52" s="34"/>
+      <x:c r="B52" s="34"/>
+      <x:c r="C52" s="34"/>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="34" t="str">
-        <x:v>protec_acceleration_z__failure_type_1</x:v>
-      </x:c>
-      <x:c r="B53" s="34" t="str">
-        <x:v>protec_acceleration_z</x:v>
-      </x:c>
-      <x:c r="C53" s="34" t="str">
-        <x:v>failure_type_1</x:v>
-      </x:c>
+      <x:c r="A53" s="34"/>
+      <x:c r="B53" s="34"/>
+      <x:c r="C53" s="34"/>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="34" t="str">
-        <x:v>protec_acceleration_z__failure_type_2</x:v>
-      </x:c>
-      <x:c r="B54" s="34" t="str">
-        <x:v>protec_acceleration_z</x:v>
-      </x:c>
-      <x:c r="C54" s="34" t="str">
-        <x:v>failure_type_2</x:v>
-      </x:c>
+      <x:c r="A54" s="34"/>
+      <x:c r="B54" s="34"/>
+      <x:c r="C54" s="34"/>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="34" t="str">
-        <x:v>protec_acceleration_z__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B55" s="34" t="str">
-        <x:v>protec_acceleration_z</x:v>
-      </x:c>
-      <x:c r="C55" s="34" t="str">
-        <x:v>failure_type_3</x:v>
-      </x:c>
+      <x:c r="A55" s="34"/>
+      <x:c r="B55" s="34"/>
+      <x:c r="C55" s="34"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re82e7b281e754d1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbc82289c878422f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2889,7 +2500,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reda44e3e968340f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8d926fc13884012"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -51890,7 +51501,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R380ce126d24d45e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda25b499aaca48c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -51929,77 +51540,37 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="34" t="str">
-        <x:v>eta_beta_initial_1</x:v>
-      </x:c>
-      <x:c r="B5" s="34" t="str">
-        <x:v>asset_failure_type_1</x:v>
-      </x:c>
-      <x:c r="C5" s="39" t="n">
-        <x:v>10000</x:v>
-      </x:c>
-      <x:c r="D5" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E5" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A5" s="34"/>
+      <x:c r="B5" s="34"/>
+      <x:c r="C5" s="39"/>
+      <x:c r="D5" s="39"/>
+      <x:c r="E5" s="38"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="34" t="str">
-        <x:v>eta_beta_initial_2</x:v>
-      </x:c>
-      <x:c r="B6" s="34" t="str">
-        <x:v>asset_failure_type_2</x:v>
-      </x:c>
-      <x:c r="C6" s="39" t="n">
-        <x:v>10000</x:v>
-      </x:c>
-      <x:c r="D6" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E6" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A6" s="34"/>
+      <x:c r="B6" s="34"/>
+      <x:c r="C6" s="39"/>
+      <x:c r="D6" s="39"/>
+      <x:c r="E6" s="38"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="34" t="str">
-        <x:v>eta_beta_initial_3</x:v>
-      </x:c>
-      <x:c r="B7" s="34" t="str">
-        <x:v>asset_failure_type_3</x:v>
-      </x:c>
-      <x:c r="C7" s="39" t="n">
-        <x:v>10000</x:v>
-      </x:c>
-      <x:c r="D7" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E7" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A7" s="34"/>
+      <x:c r="B7" s="34"/>
+      <x:c r="C7" s="39"/>
+      <x:c r="D7" s="39"/>
+      <x:c r="E7" s="38"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="34" t="str">
-        <x:v>eta_beta_initial_4</x:v>
-      </x:c>
-      <x:c r="B8" s="34" t="str">
-        <x:v>asset_failure_type_4</x:v>
-      </x:c>
-      <x:c r="C8" s="39" t="n">
-        <x:v>10000</x:v>
-      </x:c>
-      <x:c r="D8" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E8" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A8" s="34"/>
+      <x:c r="B8" s="34"/>
+      <x:c r="C8" s="39"/>
+      <x:c r="D8" s="39"/>
+      <x:c r="E8" s="38"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R072e3a161a324806"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6ef2332aff4494e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -52038,876 +51609,366 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="34" t="str">
-        <x:v>gamma_initial_1</x:v>
-      </x:c>
-      <x:c r="B5" s="34" t="str">
-        <x:v>tray_in_vqc__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C5" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D5" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E5" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A5" s="34"/>
+      <x:c r="B5" s="34"/>
+      <x:c r="C5" s="39"/>
+      <x:c r="D5" s="39"/>
+      <x:c r="E5" s="38"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="34" t="str">
-        <x:v>gamma_initial_2</x:v>
-      </x:c>
-      <x:c r="B6" s="34" t="str">
-        <x:v>tray_in_vqc__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C6" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D6" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E6" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A6" s="34"/>
+      <x:c r="B6" s="34"/>
+      <x:c r="C6" s="39"/>
+      <x:c r="D6" s="39"/>
+      <x:c r="E6" s="38"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="34" t="str">
-        <x:v>gamma_initial_3</x:v>
-      </x:c>
-      <x:c r="B7" s="34" t="str">
-        <x:v>tray_in_vqc__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C7" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D7" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E7" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A7" s="34"/>
+      <x:c r="B7" s="34"/>
+      <x:c r="C7" s="39"/>
+      <x:c r="D7" s="39"/>
+      <x:c r="E7" s="38"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="34" t="str">
-        <x:v>gamma_initial_4</x:v>
-      </x:c>
-      <x:c r="B8" s="34" t="str">
-        <x:v>tray_out_vqc__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C8" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D8" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E8" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A8" s="34"/>
+      <x:c r="B8" s="34"/>
+      <x:c r="C8" s="39"/>
+      <x:c r="D8" s="39"/>
+      <x:c r="E8" s="38"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="34" t="str">
-        <x:v>gamma_initial_5</x:v>
-      </x:c>
-      <x:c r="B9" s="34" t="str">
-        <x:v>tray_out_vqc__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C9" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D9" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E9" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A9" s="34"/>
+      <x:c r="B9" s="34"/>
+      <x:c r="C9" s="39"/>
+      <x:c r="D9" s="39"/>
+      <x:c r="E9" s="38"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="34" t="str">
-        <x:v>gamma_initial_6</x:v>
-      </x:c>
-      <x:c r="B10" s="34" t="str">
-        <x:v>tray_out_vqc__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C10" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D10" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E10" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A10" s="34"/>
+      <x:c r="B10" s="34"/>
+      <x:c r="C10" s="39"/>
+      <x:c r="D10" s="39"/>
+      <x:c r="E10" s="38"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="34" t="str">
-        <x:v>gamma_initial_7</x:v>
-      </x:c>
-      <x:c r="B11" s="34" t="str">
-        <x:v>cylinder_status_vqc__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C11" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D11" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E11" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A11" s="34"/>
+      <x:c r="B11" s="34"/>
+      <x:c r="C11" s="39"/>
+      <x:c r="D11" s="39"/>
+      <x:c r="E11" s="38"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="34" t="str">
-        <x:v>gamma_initial_8</x:v>
-      </x:c>
-      <x:c r="B12" s="34" t="str">
-        <x:v>cylinder_status_vqc__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C12" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D12" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E12" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A12" s="34"/>
+      <x:c r="B12" s="34"/>
+      <x:c r="C12" s="39"/>
+      <x:c r="D12" s="39"/>
+      <x:c r="E12" s="38"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="34" t="str">
-        <x:v>gamma_initial_9</x:v>
-      </x:c>
-      <x:c r="B13" s="34" t="str">
-        <x:v>cylinder_status_vqc__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C13" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D13" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E13" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A13" s="34"/>
+      <x:c r="B13" s="34"/>
+      <x:c r="C13" s="39"/>
+      <x:c r="D13" s="39"/>
+      <x:c r="E13" s="38"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="34" t="str">
-        <x:v>gamma_initial_10</x:v>
-      </x:c>
-      <x:c r="B14" s="34" t="str">
-        <x:v>tray_in_prep__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C14" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D14" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E14" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A14" s="34"/>
+      <x:c r="B14" s="34"/>
+      <x:c r="C14" s="39"/>
+      <x:c r="D14" s="39"/>
+      <x:c r="E14" s="38"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="34" t="str">
-        <x:v>gamma_initial_11</x:v>
-      </x:c>
-      <x:c r="B15" s="34" t="str">
-        <x:v>tray_in_prep__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C15" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D15" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E15" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A15" s="34"/>
+      <x:c r="B15" s="34"/>
+      <x:c r="C15" s="39"/>
+      <x:c r="D15" s="39"/>
+      <x:c r="E15" s="38"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="34" t="str">
-        <x:v>gamma_initial_12</x:v>
-      </x:c>
-      <x:c r="B16" s="34" t="str">
-        <x:v>tray_in_prep__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C16" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D16" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E16" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A16" s="34"/>
+      <x:c r="B16" s="34"/>
+      <x:c r="C16" s="39"/>
+      <x:c r="D16" s="39"/>
+      <x:c r="E16" s="38"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="34" t="str">
-        <x:v>gamma_initial_13</x:v>
-      </x:c>
-      <x:c r="B17" s="34" t="str">
-        <x:v>tray_out_prep__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C17" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D17" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E17" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A17" s="34"/>
+      <x:c r="B17" s="34"/>
+      <x:c r="C17" s="39"/>
+      <x:c r="D17" s="39"/>
+      <x:c r="E17" s="38"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="34" t="str">
-        <x:v>gamma_initial_14</x:v>
-      </x:c>
-      <x:c r="B18" s="34" t="str">
-        <x:v>tray_out_prep__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C18" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D18" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E18" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A18" s="34"/>
+      <x:c r="B18" s="34"/>
+      <x:c r="C18" s="39"/>
+      <x:c r="D18" s="39"/>
+      <x:c r="E18" s="38"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="34" t="str">
-        <x:v>gamma_initial_15</x:v>
-      </x:c>
-      <x:c r="B19" s="34" t="str">
-        <x:v>tray_out_prep__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C19" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D19" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E19" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A19" s="34"/>
+      <x:c r="B19" s="34"/>
+      <x:c r="C19" s="39"/>
+      <x:c r="D19" s="39"/>
+      <x:c r="E19" s="38"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="34" t="str">
-        <x:v>gamma_initial_16</x:v>
-      </x:c>
-      <x:c r="B20" s="34" t="str">
-        <x:v>cylinder_status_prep__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C20" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D20" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E20" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A20" s="34"/>
+      <x:c r="B20" s="34"/>
+      <x:c r="C20" s="39"/>
+      <x:c r="D20" s="39"/>
+      <x:c r="E20" s="38"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="34" t="str">
-        <x:v>gamma_initial_17</x:v>
-      </x:c>
-      <x:c r="B21" s="34" t="str">
-        <x:v>cylinder_status_prep__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C21" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D21" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E21" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A21" s="34"/>
+      <x:c r="B21" s="34"/>
+      <x:c r="C21" s="39"/>
+      <x:c r="D21" s="39"/>
+      <x:c r="E21" s="38"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="34" t="str">
-        <x:v>gamma_initial_18</x:v>
-      </x:c>
-      <x:c r="B22" s="34" t="str">
-        <x:v>cylinder_status_prep__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C22" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D22" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E22" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A22" s="34"/>
+      <x:c r="B22" s="34"/>
+      <x:c r="C22" s="39"/>
+      <x:c r="D22" s="39"/>
+      <x:c r="E22" s="38"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="34" t="str">
-        <x:v>gamma_initial_19</x:v>
-      </x:c>
-      <x:c r="B23" s="34" t="str">
-        <x:v>tray_in_asb1__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C23" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D23" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E23" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A23" s="34"/>
+      <x:c r="B23" s="34"/>
+      <x:c r="C23" s="39"/>
+      <x:c r="D23" s="39"/>
+      <x:c r="E23" s="38"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="34" t="str">
-        <x:v>gamma_initial_20</x:v>
-      </x:c>
-      <x:c r="B24" s="34" t="str">
-        <x:v>tray_in_asb1__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C24" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D24" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E24" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A24" s="34"/>
+      <x:c r="B24" s="34"/>
+      <x:c r="C24" s="39"/>
+      <x:c r="D24" s="39"/>
+      <x:c r="E24" s="38"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="34" t="str">
-        <x:v>gamma_initial_21</x:v>
-      </x:c>
-      <x:c r="B25" s="34" t="str">
-        <x:v>tray_in_asb1__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C25" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D25" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E25" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A25" s="34"/>
+      <x:c r="B25" s="34"/>
+      <x:c r="C25" s="39"/>
+      <x:c r="D25" s="39"/>
+      <x:c r="E25" s="38"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="34" t="str">
-        <x:v>gamma_initial_22</x:v>
-      </x:c>
-      <x:c r="B26" s="34" t="str">
-        <x:v>tray_out_asb1__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C26" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D26" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E26" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A26" s="34"/>
+      <x:c r="B26" s="34"/>
+      <x:c r="C26" s="39"/>
+      <x:c r="D26" s="39"/>
+      <x:c r="E26" s="38"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="34" t="str">
-        <x:v>gamma_initial_23</x:v>
-      </x:c>
-      <x:c r="B27" s="34" t="str">
-        <x:v>tray_out_asb1__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C27" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D27" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E27" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A27" s="34"/>
+      <x:c r="B27" s="34"/>
+      <x:c r="C27" s="39"/>
+      <x:c r="D27" s="39"/>
+      <x:c r="E27" s="38"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="34" t="str">
-        <x:v>gamma_initial_24</x:v>
-      </x:c>
-      <x:c r="B28" s="34" t="str">
-        <x:v>tray_out_asb1__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C28" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D28" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E28" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A28" s="34"/>
+      <x:c r="B28" s="34"/>
+      <x:c r="C28" s="39"/>
+      <x:c r="D28" s="39"/>
+      <x:c r="E28" s="38"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="34" t="str">
-        <x:v>gamma_initial_25</x:v>
-      </x:c>
-      <x:c r="B29" s="34" t="str">
-        <x:v>cylinder_status_asb1__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C29" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D29" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E29" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A29" s="34"/>
+      <x:c r="B29" s="34"/>
+      <x:c r="C29" s="39"/>
+      <x:c r="D29" s="39"/>
+      <x:c r="E29" s="38"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="34" t="str">
-        <x:v>gamma_initial_26</x:v>
-      </x:c>
-      <x:c r="B30" s="34" t="str">
-        <x:v>cylinder_status_asb1__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C30" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D30" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E30" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A30" s="34"/>
+      <x:c r="B30" s="34"/>
+      <x:c r="C30" s="39"/>
+      <x:c r="D30" s="39"/>
+      <x:c r="E30" s="38"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="34" t="str">
-        <x:v>gamma_initial_27</x:v>
-      </x:c>
-      <x:c r="B31" s="34" t="str">
-        <x:v>cylinder_status_asb1__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C31" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D31" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E31" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A31" s="34"/>
+      <x:c r="B31" s="34"/>
+      <x:c r="C31" s="39"/>
+      <x:c r="D31" s="39"/>
+      <x:c r="E31" s="38"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="34" t="str">
-        <x:v>gamma_initial_28</x:v>
-      </x:c>
-      <x:c r="B32" s="34" t="str">
-        <x:v>tray_in_asb2__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C32" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D32" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E32" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A32" s="34"/>
+      <x:c r="B32" s="34"/>
+      <x:c r="C32" s="39"/>
+      <x:c r="D32" s="39"/>
+      <x:c r="E32" s="38"/>
     </x:row>
     <x:row r="33">
-      <x:c r="A33" s="34" t="str">
-        <x:v>gamma_initial_29</x:v>
-      </x:c>
-      <x:c r="B33" s="34" t="str">
-        <x:v>tray_in_asb2__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C33" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D33" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E33" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A33" s="34"/>
+      <x:c r="B33" s="34"/>
+      <x:c r="C33" s="39"/>
+      <x:c r="D33" s="39"/>
+      <x:c r="E33" s="38"/>
     </x:row>
     <x:row r="34">
-      <x:c r="A34" s="34" t="str">
-        <x:v>gamma_initial_30</x:v>
-      </x:c>
-      <x:c r="B34" s="34" t="str">
-        <x:v>tray_in_asb2__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C34" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D34" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E34" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A34" s="34"/>
+      <x:c r="B34" s="34"/>
+      <x:c r="C34" s="39"/>
+      <x:c r="D34" s="39"/>
+      <x:c r="E34" s="38"/>
     </x:row>
     <x:row r="35">
-      <x:c r="A35" s="34" t="str">
-        <x:v>gamma_initial_31</x:v>
-      </x:c>
-      <x:c r="B35" s="34" t="str">
-        <x:v>tray_out_asb2__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C35" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D35" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E35" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A35" s="34"/>
+      <x:c r="B35" s="34"/>
+      <x:c r="C35" s="39"/>
+      <x:c r="D35" s="39"/>
+      <x:c r="E35" s="38"/>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="34" t="str">
-        <x:v>gamma_initial_32</x:v>
-      </x:c>
-      <x:c r="B36" s="34" t="str">
-        <x:v>tray_out_asb2__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C36" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D36" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E36" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A36" s="34"/>
+      <x:c r="B36" s="34"/>
+      <x:c r="C36" s="39"/>
+      <x:c r="D36" s="39"/>
+      <x:c r="E36" s="38"/>
     </x:row>
     <x:row r="37">
-      <x:c r="A37" s="34" t="str">
-        <x:v>gamma_initial_33</x:v>
-      </x:c>
-      <x:c r="B37" s="34" t="str">
-        <x:v>tray_out_asb2__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C37" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D37" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E37" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A37" s="34"/>
+      <x:c r="B37" s="34"/>
+      <x:c r="C37" s="39"/>
+      <x:c r="D37" s="39"/>
+      <x:c r="E37" s="38"/>
     </x:row>
     <x:row r="38">
-      <x:c r="A38" s="34" t="str">
-        <x:v>gamma_initial_34</x:v>
-      </x:c>
-      <x:c r="B38" s="34" t="str">
-        <x:v>cylinder_status_asb2__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C38" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D38" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E38" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A38" s="34"/>
+      <x:c r="B38" s="34"/>
+      <x:c r="C38" s="39"/>
+      <x:c r="D38" s="39"/>
+      <x:c r="E38" s="38"/>
     </x:row>
     <x:row r="39">
-      <x:c r="A39" s="34" t="str">
-        <x:v>gamma_initial_35</x:v>
-      </x:c>
-      <x:c r="B39" s="34" t="str">
-        <x:v>cylinder_status_asb2__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C39" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D39" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E39" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A39" s="34"/>
+      <x:c r="B39" s="34"/>
+      <x:c r="C39" s="39"/>
+      <x:c r="D39" s="39"/>
+      <x:c r="E39" s="38"/>
     </x:row>
     <x:row r="40">
-      <x:c r="A40" s="34" t="str">
-        <x:v>gamma_initial_36</x:v>
-      </x:c>
-      <x:c r="B40" s="34" t="str">
-        <x:v>cylinder_status_asb2__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C40" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D40" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E40" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A40" s="34"/>
+      <x:c r="B40" s="34"/>
+      <x:c r="C40" s="39"/>
+      <x:c r="D40" s="39"/>
+      <x:c r="E40" s="38"/>
     </x:row>
     <x:row r="41">
-      <x:c r="A41" s="34" t="str">
-        <x:v>gamma_initial_37</x:v>
-      </x:c>
-      <x:c r="B41" s="34" t="str">
-        <x:v>global_temp__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C41" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D41" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E41" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A41" s="34"/>
+      <x:c r="B41" s="34"/>
+      <x:c r="C41" s="39"/>
+      <x:c r="D41" s="39"/>
+      <x:c r="E41" s="38"/>
     </x:row>
     <x:row r="42">
-      <x:c r="A42" s="34" t="str">
-        <x:v>gamma_initial_38</x:v>
-      </x:c>
-      <x:c r="B42" s="34" t="str">
-        <x:v>global_temp__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C42" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D42" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E42" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A42" s="34"/>
+      <x:c r="B42" s="34"/>
+      <x:c r="C42" s="39"/>
+      <x:c r="D42" s="39"/>
+      <x:c r="E42" s="38"/>
     </x:row>
     <x:row r="43">
-      <x:c r="A43" s="34" t="str">
-        <x:v>gamma_initial_39</x:v>
-      </x:c>
-      <x:c r="B43" s="34" t="str">
-        <x:v>global_temp__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C43" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D43" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E43" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A43" s="34"/>
+      <x:c r="B43" s="34"/>
+      <x:c r="C43" s="39"/>
+      <x:c r="D43" s="39"/>
+      <x:c r="E43" s="38"/>
     </x:row>
     <x:row r="44">
-      <x:c r="A44" s="34" t="str">
-        <x:v>gamma_initial_40</x:v>
-      </x:c>
-      <x:c r="B44" s="34" t="str">
-        <x:v>global_hum__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C44" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D44" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E44" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A44" s="34"/>
+      <x:c r="B44" s="34"/>
+      <x:c r="C44" s="39"/>
+      <x:c r="D44" s="39"/>
+      <x:c r="E44" s="38"/>
     </x:row>
     <x:row r="45">
-      <x:c r="A45" s="34" t="str">
-        <x:v>gamma_initial_41</x:v>
-      </x:c>
-      <x:c r="B45" s="34" t="str">
-        <x:v>global_hum__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C45" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D45" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E45" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A45" s="34"/>
+      <x:c r="B45" s="34"/>
+      <x:c r="C45" s="39"/>
+      <x:c r="D45" s="39"/>
+      <x:c r="E45" s="38"/>
     </x:row>
     <x:row r="46">
-      <x:c r="A46" s="34" t="str">
-        <x:v>gamma_initial_42</x:v>
-      </x:c>
-      <x:c r="B46" s="34" t="str">
-        <x:v>global_hum__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C46" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D46" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E46" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A46" s="34"/>
+      <x:c r="B46" s="34"/>
+      <x:c r="C46" s="39"/>
+      <x:c r="D46" s="39"/>
+      <x:c r="E46" s="38"/>
     </x:row>
     <x:row r="47">
-      <x:c r="A47" s="34" t="str">
-        <x:v>gamma_initial_43</x:v>
-      </x:c>
-      <x:c r="B47" s="34" t="str">
-        <x:v>protec_acceleration_x__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C47" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D47" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E47" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A47" s="34"/>
+      <x:c r="B47" s="34"/>
+      <x:c r="C47" s="39"/>
+      <x:c r="D47" s="39"/>
+      <x:c r="E47" s="38"/>
     </x:row>
     <x:row r="48">
-      <x:c r="A48" s="34" t="str">
-        <x:v>gamma_initial_44</x:v>
-      </x:c>
-      <x:c r="B48" s="34" t="str">
-        <x:v>protec_acceleration_x__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C48" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D48" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E48" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A48" s="34"/>
+      <x:c r="B48" s="34"/>
+      <x:c r="C48" s="39"/>
+      <x:c r="D48" s="39"/>
+      <x:c r="E48" s="38"/>
     </x:row>
     <x:row r="49">
-      <x:c r="A49" s="34" t="str">
-        <x:v>gamma_initial_45</x:v>
-      </x:c>
-      <x:c r="B49" s="34" t="str">
-        <x:v>protec_acceleration_x__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C49" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D49" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E49" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A49" s="34"/>
+      <x:c r="B49" s="34"/>
+      <x:c r="C49" s="39"/>
+      <x:c r="D49" s="39"/>
+      <x:c r="E49" s="38"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="34" t="str">
-        <x:v>gamma_initial_46</x:v>
-      </x:c>
-      <x:c r="B50" s="34" t="str">
-        <x:v>protec_acceleration_y__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C50" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D50" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E50" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A50" s="34"/>
+      <x:c r="B50" s="34"/>
+      <x:c r="C50" s="39"/>
+      <x:c r="D50" s="39"/>
+      <x:c r="E50" s="38"/>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="34" t="str">
-        <x:v>gamma_initial_47</x:v>
-      </x:c>
-      <x:c r="B51" s="34" t="str">
-        <x:v>protec_acceleration_y__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C51" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D51" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E51" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A51" s="34"/>
+      <x:c r="B51" s="34"/>
+      <x:c r="C51" s="39"/>
+      <x:c r="D51" s="39"/>
+      <x:c r="E51" s="38"/>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="34" t="str">
-        <x:v>gamma_initial_48</x:v>
-      </x:c>
-      <x:c r="B52" s="34" t="str">
-        <x:v>protec_acceleration_y__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C52" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D52" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E52" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A52" s="34"/>
+      <x:c r="B52" s="34"/>
+      <x:c r="C52" s="39"/>
+      <x:c r="D52" s="39"/>
+      <x:c r="E52" s="38"/>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="34" t="str">
-        <x:v>gamma_initial_49</x:v>
-      </x:c>
-      <x:c r="B53" s="34" t="str">
-        <x:v>protec_acceleration_z__failure_type_1</x:v>
-      </x:c>
-      <x:c r="C53" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D53" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E53" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A53" s="34"/>
+      <x:c r="B53" s="34"/>
+      <x:c r="C53" s="39"/>
+      <x:c r="D53" s="39"/>
+      <x:c r="E53" s="38"/>
     </x:row>
     <x:row r="54">
-      <x:c r="A54" s="34" t="str">
-        <x:v>gamma_initial_50</x:v>
-      </x:c>
-      <x:c r="B54" s="34" t="str">
-        <x:v>protec_acceleration_z__failure_type_2</x:v>
-      </x:c>
-      <x:c r="C54" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D54" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E54" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A54" s="34"/>
+      <x:c r="B54" s="34"/>
+      <x:c r="C54" s="39"/>
+      <x:c r="D54" s="39"/>
+      <x:c r="E54" s="38"/>
     </x:row>
     <x:row r="55">
-      <x:c r="A55" s="34" t="str">
-        <x:v>gamma_initial__protec_acceleration_z__failure_type_3</x:v>
-      </x:c>
-      <x:c r="B55" s="34" t="str">
-        <x:v>protec_acceleration_z__failure_type_3</x:v>
-      </x:c>
-      <x:c r="C55" s="39" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="D55" s="39" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E55" s="38" t="n">
-        <x:v>46266</x:v>
-      </x:c>
+      <x:c r="A55" s="34"/>
+      <x:c r="B55" s="34"/>
+      <x:c r="C55" s="39"/>
+      <x:c r="D55" s="39"/>
+      <x:c r="E55" s="38"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb254d3fab0ef4f6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4d9367f4c4f4d92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -52930,7 +51991,7 @@
     </x:row>
     <x:row r="2" ht="18.75" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -52944,36 +52005,36 @@
     </x:row>
     <x:row r="4" ht="26.100000381469727" customHeight="1">
       <x:c r="A4" s="3" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="s">
+      <x:c r="C4" s="3" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="C4" s="3" t="s">
+      <x:c r="D4" s="3" t="s">
         <x:v>20</x:v>
-      </x:c>
-      <x:c r="D4" s="3" t="s">
-        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="18.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="B5" s="3" t="s">
+      <x:c r="C5" s="3" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="C5" s="3" t="s">
+      <x:c r="D5" s="11" t="s">
         <x:v>24</x:v>
-      </x:c>
-      <x:c r="D5" s="11" t="s">
-        <x:v>25</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c7d181fb1684d5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53a7b41f95cd40af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53158,9 +52219,7 @@
       <x:c r="E10" s="38" t="n">
         <x:v>46032.416666666664</x:v>
       </x:c>
-      <x:c r="F10" s="34" t="str">
-        <x:v>asset_failure_type_4</x:v>
-      </x:c>
+      <x:c r="F10" s="34"/>
       <x:c r="G10" s="38" t="n">
         <x:v>46032.381944444445</x:v>
       </x:c>
@@ -53174,7 +52233,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff13f6f32307425c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a33f09779744f51"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53589,7 +52648,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3b2320f500c4037"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf44ddc35374b48e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53608,7 +52667,7 @@
     </x:row>
     <x:row r="2" ht="18.75" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
     </x:row>
@@ -53618,64 +52677,64 @@
     </x:row>
     <x:row r="4" ht="26.100000381469727" customHeight="1">
       <x:c r="A4" s="3" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
         <x:v>27</x:v>
-      </x:c>
-      <x:c r="B4" s="3" t="s">
-        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="18.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
         <x:v>29</x:v>
-      </x:c>
-      <x:c r="B5" s="3" t="s">
-        <x:v>30</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="18.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="s">
         <x:v>31</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="s">
-        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="18.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="s">
         <x:v>33</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="s">
-        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="18.75" customHeight="1">
       <x:c r="A8" s="3" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="s">
         <x:v>35</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="s">
-        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="18.75" customHeight="1">
       <x:c r="A9" s="3" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="s">
         <x:v>37</x:v>
-      </x:c>
-      <x:c r="B9" s="3" t="s">
-        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="18.75" customHeight="1">
       <x:c r="A10" s="3" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="s">
         <x:v>39</x:v>
-      </x:c>
-      <x:c r="B10" s="3" t="s">
-        <x:v>40</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdafc8a382cb74ee5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfde3fd8039c54f91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53696,7 +52755,7 @@
     </x:row>
     <x:row r="2" ht="18.75" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="18"/>
@@ -53708,21 +52767,21 @@
     </x:row>
     <x:row r="4" ht="26.100000381469727" customHeight="1">
       <x:c r="A4" s="3" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="s">
+      <x:c r="C4" s="18" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="C4" s="18" t="s">
-        <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="18.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
         <x:v>45</x:v>
-      </x:c>
-      <x:c r="B5" s="3" t="s">
-        <x:v>46</x:v>
       </x:c>
       <x:c r="C5" s="23">
         <x:v>19</x:v>
@@ -53730,10 +52789,10 @@
     </x:row>
     <x:row r="6" ht="18.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="s">
         <x:v>47</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="s">
-        <x:v>48</x:v>
       </x:c>
       <x:c r="C6" s="23">
         <x:v>19</x:v>
@@ -53741,10 +52800,10 @@
     </x:row>
     <x:row r="7" ht="18.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="s">
         <x:v>49</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="s">
-        <x:v>50</x:v>
       </x:c>
       <x:c r="C7" s="23">
         <x:v>19</x:v>
@@ -53752,10 +52811,10 @@
     </x:row>
     <x:row r="8" ht="18.75" customHeight="1">
       <x:c r="A8" s="3" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="s">
         <x:v>51</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="s">
-        <x:v>52</x:v>
       </x:c>
       <x:c r="C8" s="23">
         <x:v>19</x:v>
@@ -53764,7 +52823,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fb3468a23f242e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R714c25fd95a64d9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53787,7 +52846,7 @@
     </x:row>
     <x:row r="2" ht="18.75" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -53801,84 +52860,84 @@
     </x:row>
     <x:row r="4" ht="26.100000381469727" customHeight="1">
       <x:c r="A4" s="3" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
         <x:v>54</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="s">
+      <x:c r="C4" s="3" t="s">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="C4" s="3" t="s">
+      <x:c r="D4" s="3" t="s">
         <x:v>56</x:v>
-      </x:c>
-      <x:c r="D4" s="3" t="s">
-        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="18.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
         <x:v>58</x:v>
-      </x:c>
-      <x:c r="B5" s="3" t="s">
-        <x:v>59</x:v>
       </x:c>
       <x:c r="C5" s="1"/>
       <x:c r="D5" s="1"/>
     </x:row>
     <x:row r="6" ht="18.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="s">
         <x:v>60</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="s">
-        <x:v>61</x:v>
       </x:c>
       <x:c r="C6" s="1"/>
       <x:c r="D6" s="1"/>
     </x:row>
     <x:row r="7" ht="18.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="s">
         <x:v>62</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="s">
-        <x:v>63</x:v>
       </x:c>
       <x:c r="C7" s="1"/>
       <x:c r="D7" s="1"/>
     </x:row>
     <x:row r="8" ht="18.75" customHeight="1">
       <x:c r="A8" s="3" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="s">
         <x:v>64</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="s">
-        <x:v>65</x:v>
       </x:c>
       <x:c r="C8" s="1"/>
       <x:c r="D8" s="1"/>
     </x:row>
     <x:row r="9" ht="18.75" customHeight="1">
       <x:c r="A9" s="3" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="C9" s="1"/>
       <x:c r="D9" s="1"/>
     </x:row>
     <x:row r="10" ht="18.75" customHeight="1">
       <x:c r="A10" s="3" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="s">
         <x:v>67</x:v>
-      </x:c>
-      <x:c r="B10" s="3" t="s">
-        <x:v>68</x:v>
       </x:c>
       <x:c r="C10" s="1"/>
       <x:c r="D10" s="1"/>
     </x:row>
     <x:row r="11" ht="18.75" customHeight="1">
       <x:c r="A11" s="3" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="s">
         <x:v>69</x:v>
-      </x:c>
-      <x:c r="B11" s="3" t="s">
-        <x:v>70</x:v>
       </x:c>
       <x:c r="C11" s="1"/>
       <x:c r="D11" s="1"/>
@@ -53886,7 +52945,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01b355486dea4b6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda2e1204d9c64f7b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -53911,7 +52970,7 @@
     </x:row>
     <x:row r="2" ht="18.75" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -53927,82 +52986,82 @@
     </x:row>
     <x:row r="4" ht="26.100000381469727" customHeight="1">
       <x:c r="A4" s="3" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="s">
+      <x:c r="C4" s="3" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C4" s="3" t="s">
+      <x:c r="D4" s="3" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="D4" s="3" t="s">
+      <x:c r="E4" s="3" t="s">
         <x:v>75</x:v>
-      </x:c>
-      <x:c r="E4" s="3" t="s">
-        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="18.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="B5" s="3" t="s">
+      <x:c r="C5" s="3" t="s">
         <x:v>78</x:v>
-      </x:c>
-      <x:c r="C5" s="3" t="s">
-        <x:v>79</x:v>
       </x:c>
       <x:c r="D5" s="1"/>
       <x:c r="E5" s="1"/>
     </x:row>
     <x:row r="6" ht="18.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="B6" s="3" t="s">
-        <x:v>81</x:v>
-      </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>79</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="D6" s="1"/>
       <x:c r="E6" s="1"/>
     </x:row>
     <x:row r="7" ht="18.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="s">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="B7" s="3" t="s">
+      <x:c r="C7" s="3" t="s">
         <x:v>83</x:v>
-      </x:c>
-      <x:c r="C7" s="3" t="s">
-        <x:v>84</x:v>
       </x:c>
       <x:c r="D7" s="1"/>
       <x:c r="E7" s="1"/>
     </x:row>
     <x:row r="8" ht="18.75" customHeight="1">
       <x:c r="A8" s="3" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="s">
         <x:v>85</x:v>
       </x:c>
-      <x:c r="B8" s="3" t="s">
+      <x:c r="C8" s="3" t="s">
         <x:v>86</x:v>
-      </x:c>
-      <x:c r="C8" s="3" t="s">
-        <x:v>87</x:v>
       </x:c>
       <x:c r="D8" s="1"/>
       <x:c r="E8" s="1"/>
     </x:row>
     <x:row r="9" ht="18.75" customHeight="1">
       <x:c r="A9" s="1" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="B9" s="1" t="s">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="B9" s="1" t="s">
+      <x:c r="C9" s="1" t="s">
         <x:v>89</x:v>
-      </x:c>
-      <x:c r="C9" s="1" t="s">
-        <x:v>90</x:v>
       </x:c>
       <x:c r="D9" s="1"/>
       <x:c r="E9" s="1"/>
@@ -54010,7 +53069,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9bd50c09a484306"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a70a8adf48b4107"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54037,7 +53096,7 @@
     </x:row>
     <x:row r="2" ht="18.75" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>91</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="18"/>
@@ -54055,30 +53114,30 @@
     </x:row>
     <x:row r="4" ht="26.100000381469727" customHeight="1">
       <x:c r="A4" s="3" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="s">
+      <x:c r="C4" s="18" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="C4" s="18" t="s">
+      <x:c r="D4" s="18" t="s">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="D4" s="18" t="s">
+      <x:c r="E4" s="3" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="F4" s="3" t="s">
         <x:v>95</x:v>
-      </x:c>
-      <x:c r="E4" s="3" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="F4" s="3" t="s">
-        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="18.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>96</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
         <x:v>97</x:v>
-      </x:c>
-      <x:c r="B5" s="3" t="s">
-        <x:v>98</x:v>
       </x:c>
       <x:c r="C5" s="9">
         <x:v>1</x:v>
@@ -54087,16 +53146,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>77</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="F5" s="20"/>
     </x:row>
     <x:row r="6" ht="18.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="s">
         <x:v>99</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="s">
-        <x:v>100</x:v>
       </x:c>
       <x:c r="C6" s="9">
         <x:v>1</x:v>
@@ -54105,16 +53164,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="3" t="s">
-        <x:v>80</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="F6" s="20"/>
     </x:row>
     <x:row r="7" ht="18.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="s">
         <x:v>101</x:v>
-      </x:c>
-      <x:c r="B7" s="3" t="s">
-        <x:v>102</x:v>
       </x:c>
       <x:c r="C7" s="9">
         <x:v>50</x:v>
@@ -54123,16 +53182,16 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="3" t="s">
-        <x:v>82</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="F7" s="20"/>
     </x:row>
     <x:row r="8" ht="18.75" customHeight="1">
       <x:c r="A8" s="3" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="s">
         <x:v>103</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="s">
-        <x:v>104</x:v>
       </x:c>
       <x:c r="C8" s="9">
         <x:v>90</x:v>
@@ -54141,16 +53200,16 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="E8" s="3" t="s">
-        <x:v>85</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="F8" s="20"/>
     </x:row>
     <x:row r="9" ht="18.75" customHeight="1">
       <x:c r="A9" s="1" t="s">
-        <x:v>105</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B9" s="1" t="s">
-        <x:v>105</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="C9" s="21">
         <x:v>2000</x:v>
@@ -54159,14 +53218,14 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="1" t="s">
-        <x:v>88</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="F9" s="1"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e2c2165726a41ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50fdf81484db40ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54197,7 +53256,7 @@
     </x:row>
     <x:row r="2" ht="18.75" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>106</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -54219,42 +53278,42 @@
     </x:row>
     <x:row r="4" ht="26.100000381469727" customHeight="1">
       <x:c r="A4" s="3" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="s">
+      <x:c r="C4" s="3" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="D4" s="3" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="E4" s="13" t="s">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="C4" s="3" t="s">
-        <x:v>92</x:v>
-      </x:c>
-      <x:c r="D4" s="3" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="E4" s="13" t="s">
+      <x:c r="F4" s="3" t="s">
         <x:v>109</x:v>
       </x:c>
-      <x:c r="F4" s="3" t="s">
+      <x:c r="G4" s="3" t="s">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="G4" s="3" t="s">
+      <x:c r="H4" s="3" t="s">
         <x:v>111</x:v>
-      </x:c>
-      <x:c r="H4" s="3" t="s">
-        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="18.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="B5" s="3" t="s">
-        <x:v>114</x:v>
-      </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E5" s="9">
         <x:v>0.5</x:v>
@@ -54262,21 +53321,21 @@
       <x:c r="F5" s="1"/>
       <x:c r="G5" s="1"/>
       <x:c r="H5" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="18.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
+        <x:v>115</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="s">
         <x:v>116</x:v>
       </x:c>
-      <x:c r="B6" s="3" t="s">
-        <x:v>117</x:v>
-      </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D6" s="3" t="s">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E6" s="9">
         <x:v>0.5</x:v>
@@ -54284,21 +53343,21 @@
       <x:c r="F6" s="1"/>
       <x:c r="G6" s="1"/>
       <x:c r="H6" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="18.75" customHeight="1">
       <x:c r="A7" s="3" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="B7" s="3" t="s">
         <x:v>118</x:v>
       </x:c>
-      <x:c r="B7" s="3" t="s">
-        <x:v>119</x:v>
-      </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>97</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D7" s="3" t="s">
-        <x:v>58</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E7" s="9">
         <x:v>0.5</x:v>
@@ -54306,21 +53365,21 @@
       <x:c r="F7" s="1"/>
       <x:c r="G7" s="1"/>
       <x:c r="H7" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="18.75" customHeight="1">
       <x:c r="A8" s="3" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="B8" s="3" t="s">
-        <x:v>121</x:v>
-      </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D8" s="3" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E8" s="9">
         <x:v>0.5</x:v>
@@ -54328,21 +53387,21 @@
       <x:c r="F8" s="1"/>
       <x:c r="G8" s="1"/>
       <x:c r="H8" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="18.75" customHeight="1">
       <x:c r="A9" s="3" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="B9" s="3" t="s">
         <x:v>122</x:v>
       </x:c>
-      <x:c r="B9" s="3" t="s">
-        <x:v>123</x:v>
-      </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E9" s="9">
         <x:v>0.5</x:v>
@@ -54350,21 +53409,21 @@
       <x:c r="F9" s="1"/>
       <x:c r="G9" s="1"/>
       <x:c r="H9" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="18.75" customHeight="1">
       <x:c r="A10" s="3" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="s">
         <x:v>124</x:v>
       </x:c>
-      <x:c r="B10" s="3" t="s">
-        <x:v>125</x:v>
-      </x:c>
       <x:c r="C10" s="3" t="s">
-        <x:v>97</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D10" s="3" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E10" s="9">
         <x:v>0.5</x:v>
@@ -54372,21 +53431,21 @@
       <x:c r="F10" s="1"/>
       <x:c r="G10" s="1"/>
       <x:c r="H10" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="18.75" customHeight="1">
       <x:c r="A11" s="3" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="B11" s="3" t="s">
-        <x:v>127</x:v>
-      </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D11" s="3" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E11" s="9">
         <x:v>0.5</x:v>
@@ -54394,21 +53453,21 @@
       <x:c r="F11" s="1"/>
       <x:c r="G11" s="1"/>
       <x:c r="H11" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="18.75" customHeight="1">
       <x:c r="A12" s="3" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="B12" s="3" t="s">
         <x:v>128</x:v>
       </x:c>
-      <x:c r="B12" s="3" t="s">
-        <x:v>129</x:v>
-      </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E12" s="9">
         <x:v>0.5</x:v>
@@ -54416,21 +53475,21 @@
       <x:c r="F12" s="1"/>
       <x:c r="G12" s="1"/>
       <x:c r="H12" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="18.75" customHeight="1">
       <x:c r="A13" s="3" t="s">
+        <x:v>129</x:v>
+      </x:c>
+      <x:c r="B13" s="3" t="s">
         <x:v>130</x:v>
       </x:c>
-      <x:c r="B13" s="3" t="s">
-        <x:v>131</x:v>
-      </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>97</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E13" s="9">
         <x:v>0.5</x:v>
@@ -54438,21 +53497,21 @@
       <x:c r="F13" s="1"/>
       <x:c r="G13" s="1"/>
       <x:c r="H13" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="18.75" customHeight="1">
       <x:c r="A14" s="3" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="s">
         <x:v>132</x:v>
       </x:c>
-      <x:c r="B14" s="3" t="s">
-        <x:v>133</x:v>
-      </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E14" s="9">
         <x:v>0.5</x:v>
@@ -54460,21 +53519,21 @@
       <x:c r="F14" s="1"/>
       <x:c r="G14" s="1"/>
       <x:c r="H14" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="18.75" customHeight="1">
       <x:c r="A15" s="3" t="s">
+        <x:v>133</x:v>
+      </x:c>
+      <x:c r="B15" s="3" t="s">
         <x:v>134</x:v>
       </x:c>
-      <x:c r="B15" s="3" t="s">
-        <x:v>135</x:v>
-      </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>99</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E15" s="9">
         <x:v>0.5</x:v>
@@ -54482,21 +53541,21 @@
       <x:c r="F15" s="1"/>
       <x:c r="G15" s="1"/>
       <x:c r="H15" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="18.75" customHeight="1">
       <x:c r="A16" s="3" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="B16" s="3" t="s">
         <x:v>136</x:v>
       </x:c>
-      <x:c r="B16" s="3" t="s">
-        <x:v>137</x:v>
-      </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>97</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E16" s="9">
         <x:v>0.5</x:v>
@@ -54504,21 +53563,21 @@
       <x:c r="F16" s="1"/>
       <x:c r="G16" s="1"/>
       <x:c r="H16" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="18.75" customHeight="1">
       <x:c r="A17" s="3" t="s">
-        <x:v>138</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
-        <x:v>138</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>101</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E17" s="9">
         <x:v>0.5</x:v>
@@ -54526,21 +53585,21 @@
       <x:c r="F17" s="1"/>
       <x:c r="G17" s="1"/>
       <x:c r="H17" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="18.75" customHeight="1">
       <x:c r="A18" s="3" t="s">
-        <x:v>139</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
-        <x:v>139</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>103</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E18" s="9">
         <x:v>0.5</x:v>
@@ -54548,21 +53607,21 @@
       <x:c r="F18" s="1"/>
       <x:c r="G18" s="1"/>
       <x:c r="H18" s="3" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="18.75" customHeight="1">
       <x:c r="A19" s="1" t="s">
-        <x:v>140</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B19" s="1" t="s">
-        <x:v>140</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="C19" s="1" t="s">
-        <x:v>105</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="D19" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E19" s="15">
         <x:v>0.1</x:v>
@@ -54570,21 +53629,21 @@
       <x:c r="F19" s="1"/>
       <x:c r="G19" s="1"/>
       <x:c r="H19" s="1" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="18.75" customHeight="1">
       <x:c r="A20" s="1" t="s">
-        <x:v>141</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="B20" s="1" t="s">
-        <x:v>141</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C20" s="1" t="s">
-        <x:v>105</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="D20" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E20" s="15">
         <x:v>0.1</x:v>
@@ -54592,21 +53651,21 @@
       <x:c r="F20" s="1"/>
       <x:c r="G20" s="1"/>
       <x:c r="H20" s="1" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="18.75" customHeight="1">
       <x:c r="A21" s="1" t="s">
-        <x:v>142</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="B21" s="1" t="s">
-        <x:v>142</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="C21" s="1" t="s">
-        <x:v>105</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="D21" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E21" s="15">
         <x:v>0.1</x:v>
@@ -54614,13 +53673,13 @@
       <x:c r="F21" s="1"/>
       <x:c r="G21" s="1"/>
       <x:c r="H21" s="1" t="s">
-        <x:v>115</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68491aba3fe844b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd73b212d48ee4c4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54645,7 +53704,7 @@
     </x:row>
     <x:row r="2" ht="18.75" customHeight="1">
       <x:c r="A2" s="2" t="s">
-        <x:v>143</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -54661,38 +53720,38 @@
     </x:row>
     <x:row r="4" ht="26.100000381469727" customHeight="1">
       <x:c r="A4" s="3" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
         <x:v>144</x:v>
       </x:c>
-      <x:c r="B4" s="3" t="s">
+      <x:c r="C4" s="3" t="s">
         <x:v>145</x:v>
       </x:c>
-      <x:c r="C4" s="3" t="s">
+      <x:c r="D4" s="3" t="s">
         <x:v>146</x:v>
       </x:c>
-      <x:c r="D4" s="3" t="s">
+      <x:c r="E4" s="3" t="s">
         <x:v>147</x:v>
-      </x:c>
-      <x:c r="E4" s="3" t="s">
-        <x:v>148</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="18.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>148</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
         <x:v>149</x:v>
-      </x:c>
-      <x:c r="B5" s="3" t="s">
-        <x:v>150</x:v>
       </x:c>
       <x:c r="C5" s="1"/>
       <x:c r="D5" s="1"/>
       <x:c r="E5" s="11" t="s">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56231d50002b42ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d5b97db01594600"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>